<commit_message>
update: dataprep - em andamento
</commit_message>
<xml_diff>
--- a/data/df.xlsx
+++ b/data/df.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e4b858b1fb629067/Documentos/health_outcomes_workers/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{20996458-E3AA-49DC-9C0B-286648A68FF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F4A72AE0-104E-4E22-B80A-A63DA2716995}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{20996458-E3AA-49DC-9C0B-286648A68FF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C6E2323C-831E-4684-835A-1C9EE21762B7}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="19440" windowHeight="14880" xr2:uid="{4BC9F0FE-87DC-E54F-A84A-606F68B4F797}"/>
   </bookViews>
@@ -455,9 +455,6 @@
     <t>hgs_esq</t>
   </si>
   <si>
-    <t>cintura_quadril_ratio</t>
-  </si>
-  <si>
     <t>who1</t>
   </si>
   <si>
@@ -675,6 +672,9 @@
   </si>
   <si>
     <t>pad</t>
+  </si>
+  <si>
+    <t>cintura_altura_ratio</t>
   </si>
 </sst>
 </file>
@@ -1181,28 +1181,28 @@
         <v>118</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="L1" s="2" t="s">
         <v>119</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="N1" s="2" t="s">
         <v>120</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="P1" s="2" t="s">
         <v>121</v>
       </c>
       <c r="Q1" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="R1" s="2" t="s">
         <v>165</v>
-      </c>
-      <c r="R1" s="2" t="s">
-        <v>166</v>
       </c>
       <c r="S1" s="2" t="s">
         <v>122</v>
@@ -1238,91 +1238,91 @@
         <v>131</v>
       </c>
       <c r="AD1" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="AE1" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="AE1" s="2" t="s">
+      <c r="AF1" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="AF1" s="2" t="s">
+      <c r="AG1" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="AG1" s="2" t="s">
+      <c r="AH1" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="AH1" s="2" t="s">
+      <c r="AI1" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="AI1" s="2" t="s">
+      <c r="AJ1" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="AJ1" s="2" t="s">
+      <c r="AK1" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="AK1" s="2" t="s">
+      <c r="AL1" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="AL1" s="2" t="s">
+      <c r="AM1" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="AM1" s="2" t="s">
+      <c r="AN1" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="AN1" s="2" t="s">
+      <c r="AO1" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="AO1" s="2" t="s">
+      <c r="AP1" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="AP1" s="2" t="s">
+      <c r="AQ1" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="AQ1" s="2" t="s">
+      <c r="AR1" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="AR1" s="2" t="s">
+      <c r="AS1" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="AS1" s="2" t="s">
+      <c r="AT1" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="AT1" s="2" t="s">
+      <c r="AU1" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="AU1" s="2" t="s">
+      <c r="AV1" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="AV1" s="2" t="s">
+      <c r="AW1" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="AW1" s="2" t="s">
+      <c r="AX1" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="AX1" s="2" t="s">
+      <c r="AY1" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="AY1" s="2" t="s">
+      <c r="AZ1" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="AZ1" s="2" t="s">
+      <c r="BA1" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="BA1" s="2" t="s">
+      <c r="BB1" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="BB1" s="2" t="s">
+      <c r="BC1" s="2" t="s">
         <v>163</v>
-      </c>
-      <c r="BC1" s="2" t="s">
-        <v>164</v>
       </c>
       <c r="BD1" s="2" t="s">
         <v>132</v>
       </c>
       <c r="BE1" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="BF1" s="2" t="s">
         <v>167</v>
-      </c>
-      <c r="BF1" s="2" t="s">
-        <v>168</v>
       </c>
       <c r="BG1" s="2" t="s">
         <v>133</v>
@@ -1334,10 +1334,10 @@
         <v>135</v>
       </c>
       <c r="BJ1" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="BK1" s="1" t="s">
         <v>210</v>
-      </c>
-      <c r="BK1" s="1" t="s">
-        <v>211</v>
       </c>
       <c r="BL1" s="2" t="s">
         <v>136</v>
@@ -1346,21 +1346,21 @@
         <v>137</v>
       </c>
       <c r="BN1" s="2" t="s">
-        <v>138</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A2" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B2" s="3">
         <v>34</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>28</v>
@@ -1378,13 +1378,13 @@
         <v>30</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="K2" s="3">
         <v>1</v>
       </c>
       <c r="L2" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M2" s="6">
         <v>40</v>
@@ -1432,7 +1432,7 @@
         <v>53</v>
       </c>
       <c r="AC2" s="7" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AD2" s="7">
         <v>5</v>
@@ -1549,16 +1549,16 @@
     </row>
     <row r="3" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A3" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B3" s="3">
         <v>59</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>28</v>
@@ -1576,13 +1576,13 @@
         <v>32</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="K3" s="4">
         <v>2</v>
       </c>
       <c r="L3" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M3" s="4">
         <v>56</v>
@@ -1633,7 +1633,7 @@
         <v>53</v>
       </c>
       <c r="AC3" s="7" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="AD3" s="7">
         <v>5</v>
@@ -1750,19 +1750,19 @@
     </row>
     <row r="4" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A4" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B4" s="3">
         <v>27</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>33</v>
@@ -1777,13 +1777,13 @@
         <v>35</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="K4" s="3">
         <v>1</v>
       </c>
       <c r="L4" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M4" s="3">
         <v>44</v>
@@ -1831,10 +1831,10 @@
         <v>53</v>
       </c>
       <c r="AB4" s="7" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="AC4" s="7" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AD4" s="7">
         <v>3</v>
@@ -1951,16 +1951,16 @@
     </row>
     <row r="5" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A5" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B5" s="3">
         <v>40</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>28</v>
@@ -1978,13 +1978,13 @@
         <v>35</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="K5" s="3">
         <v>1</v>
       </c>
       <c r="L5" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M5" s="3">
         <v>45</v>
@@ -2035,7 +2035,7 @@
         <v>53</v>
       </c>
       <c r="AC5" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AD5" s="7">
         <v>5</v>
@@ -2152,16 +2152,16 @@
     </row>
     <row r="6" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A6" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B6" s="3">
         <v>23</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>28</v>
@@ -2179,13 +2179,13 @@
         <v>40</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="K6" s="3">
         <v>2</v>
       </c>
       <c r="L6" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M6" s="3">
         <v>45</v>
@@ -2233,7 +2233,7 @@
         <v>53</v>
       </c>
       <c r="AC6" s="7" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AD6" s="7">
         <v>5</v>
@@ -2350,19 +2350,19 @@
     </row>
     <row r="7" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A7" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B7" s="3">
         <v>65</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>29</v>
@@ -2377,13 +2377,13 @@
         <v>76</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="K7" s="3">
         <v>2</v>
       </c>
       <c r="L7" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M7" s="3">
         <v>44</v>
@@ -2428,10 +2428,10 @@
         <v>54</v>
       </c>
       <c r="AB7" s="7" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="AC7" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AD7" s="7">
         <v>4</v>
@@ -2548,19 +2548,19 @@
     </row>
     <row r="8" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A8" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B8" s="3">
         <v>54</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F8" s="3" t="s">
         <v>29</v>
@@ -2575,13 +2575,13 @@
         <v>35</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="K8" s="3">
         <v>5</v>
       </c>
       <c r="L8" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M8" s="3">
         <v>60</v>
@@ -2629,7 +2629,7 @@
         <v>54</v>
       </c>
       <c r="AB8" s="7" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="AC8" s="7"/>
       <c r="AD8" s="7">
@@ -2747,19 +2747,19 @@
     </row>
     <row r="9" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A9" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B9" s="3">
         <v>49</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="F9" s="3" t="s">
         <v>29</v>
@@ -2774,13 +2774,13 @@
         <v>82</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="K9" s="3">
         <v>2</v>
       </c>
       <c r="L9" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M9" s="3">
         <v>45</v>
@@ -2828,10 +2828,10 @@
         <v>54</v>
       </c>
       <c r="AB9" s="7" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="AC9" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AD9" s="7">
         <v>5</v>
@@ -2948,16 +2948,16 @@
     </row>
     <row r="10" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A10" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B10" s="3">
         <v>27</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>28</v>
@@ -2975,11 +2975,11 @@
         <v>49</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="K10" s="3"/>
       <c r="L10" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M10" s="3">
         <v>50</v>
@@ -3027,7 +3027,7 @@
         <v>53</v>
       </c>
       <c r="AC10" s="7" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="AD10" s="7">
         <v>5</v>
@@ -3144,16 +3144,16 @@
     </row>
     <row r="11" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A11" s="3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B11" s="3">
         <v>55</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>28</v>
@@ -3171,11 +3171,11 @@
         <v>38</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="K11" s="3"/>
       <c r="L11" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M11" s="3">
         <v>40</v>
@@ -3220,10 +3220,10 @@
         <v>54</v>
       </c>
       <c r="AB11" s="7" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="AC11" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AD11" s="7">
         <v>5</v>
@@ -3340,16 +3340,16 @@
     </row>
     <row r="12" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A12" s="3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B12" s="3">
         <v>34</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>48</v>
@@ -3367,13 +3367,13 @@
         <v>98</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="K12" s="3">
         <v>1</v>
       </c>
       <c r="L12" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M12" s="3">
         <v>35</v>
@@ -3421,10 +3421,10 @@
         <v>54</v>
       </c>
       <c r="AB12" s="7" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="AC12" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AD12" s="7">
         <v>4</v>
@@ -3541,19 +3541,19 @@
     </row>
     <row r="13" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A13" s="3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B13" s="3">
         <v>32</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F13" s="3" t="s">
         <v>29</v>
@@ -3568,13 +3568,13 @@
         <v>99</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="K13" s="3">
         <v>1</v>
       </c>
       <c r="L13" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M13" s="3">
         <v>35</v>
@@ -3625,7 +3625,7 @@
         <v>53</v>
       </c>
       <c r="AC13" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AD13" s="7">
         <v>5</v>
@@ -3742,19 +3742,19 @@
     </row>
     <row r="14" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A14" s="3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B14" s="3">
         <v>51</v>
       </c>
       <c r="C14" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="D14" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="D14" s="3" t="s">
-        <v>173</v>
-      </c>
       <c r="E14" s="3" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="F14" s="3" t="s">
         <v>29</v>
@@ -3769,11 +3769,11 @@
         <v>100</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="K14" s="3"/>
       <c r="L14" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M14" s="3">
         <v>74</v>
@@ -3824,7 +3824,7 @@
         <v>53</v>
       </c>
       <c r="AC14" s="7" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="AD14" s="7">
         <v>5</v>
@@ -3941,19 +3941,19 @@
     </row>
     <row r="15" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A15" s="3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B15" s="3">
         <v>55</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F15" s="3" t="s">
         <v>29</v>
@@ -3968,11 +3968,11 @@
         <v>101</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="K15" s="3"/>
       <c r="L15" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M15" s="3">
         <v>30</v>
@@ -4017,10 +4017,10 @@
         <v>53</v>
       </c>
       <c r="AB15" s="7" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="AC15" s="7" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AD15" s="7">
         <v>3</v>
@@ -4137,16 +4137,16 @@
     </row>
     <row r="16" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A16" s="3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B16" s="3">
         <v>31</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>28</v>
@@ -4164,13 +4164,13 @@
         <v>27</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="K16" s="3">
         <v>7</v>
       </c>
       <c r="L16" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M16" s="3">
         <v>35</v>
@@ -4218,7 +4218,7 @@
         <v>53</v>
       </c>
       <c r="AC16" s="7" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="AD16" s="7">
         <v>3</v>
@@ -4335,16 +4335,16 @@
     </row>
     <row r="17" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A17" s="3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B17" s="3">
         <v>28</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E17" s="3" t="s">
         <v>48</v>
@@ -4362,11 +4362,11 @@
         <v>103</v>
       </c>
       <c r="J17" s="3" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="K17" s="3"/>
       <c r="L17" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M17" s="3">
         <v>70</v>
@@ -4417,7 +4417,7 @@
         <v>53</v>
       </c>
       <c r="AC17" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AD17" s="7">
         <v>4</v>
@@ -4534,16 +4534,16 @@
     </row>
     <row r="18" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A18" s="3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B18" s="3">
         <v>32</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="E18" s="3" t="s">
         <v>48</v>
@@ -4561,11 +4561,11 @@
         <v>39</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="K18" s="3"/>
       <c r="L18" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M18" s="3">
         <v>40</v>
@@ -4616,7 +4616,7 @@
         <v>53</v>
       </c>
       <c r="AC18" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AD18" s="7">
         <v>4</v>
@@ -4733,19 +4733,19 @@
     </row>
     <row r="19" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A19" s="3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B19" s="3">
         <v>63</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F19" s="3" t="s">
         <v>29</v>
@@ -4760,13 +4760,13 @@
         <v>35</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="K19" s="3">
         <v>1</v>
       </c>
       <c r="L19" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M19" s="3">
         <v>30</v>
@@ -4817,7 +4817,7 @@
         <v>53</v>
       </c>
       <c r="AC19" s="7" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="AD19" s="7">
         <v>2</v>
@@ -4934,16 +4934,16 @@
     </row>
     <row r="20" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A20" s="3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B20" s="3">
         <v>71</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>28</v>
@@ -4961,11 +4961,11 @@
         <v>105</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="K20" s="3"/>
       <c r="L20" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M20" s="3">
         <v>40</v>
@@ -5013,10 +5013,10 @@
         <v>54</v>
       </c>
       <c r="AB20" s="7" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="AC20" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AD20" s="7">
         <v>4</v>
@@ -5133,19 +5133,19 @@
     </row>
     <row r="21" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A21" s="3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B21" s="3">
         <v>44</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F21" s="3" t="s">
         <v>29</v>
@@ -5160,13 +5160,13 @@
         <v>106</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="K21" s="3">
         <v>1</v>
       </c>
       <c r="L21" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M21" s="3">
         <v>40</v>
@@ -5217,7 +5217,7 @@
         <v>53</v>
       </c>
       <c r="AC21" s="7" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AD21" s="7">
         <v>3</v>
@@ -5334,16 +5334,16 @@
     </row>
     <row r="22" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A22" s="3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B22" s="3">
         <v>67</v>
       </c>
       <c r="C22" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="D22" s="3" t="s">
         <v>172</v>
-      </c>
-      <c r="D22" s="3" t="s">
-        <v>173</v>
       </c>
       <c r="E22" s="3" t="s">
         <v>107</v>
@@ -5361,11 +5361,11 @@
         <v>47</v>
       </c>
       <c r="J22" s="3" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="K22" s="3"/>
       <c r="L22" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M22" s="3">
         <v>40</v>
@@ -5407,13 +5407,13 @@
         <v>21</v>
       </c>
       <c r="AA22" s="3" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="AB22" s="7" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="AC22" s="7" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AD22" s="7">
         <v>5</v>
@@ -5530,19 +5530,19 @@
     </row>
     <row r="23" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A23" s="3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B23" s="3">
         <v>38</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F23" s="3" t="s">
         <v>33</v>
@@ -5557,13 +5557,13 @@
         <v>100</v>
       </c>
       <c r="J23" s="3" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="K23" s="3">
         <v>3</v>
       </c>
       <c r="L23" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M23" s="3">
         <v>35</v>
@@ -5611,7 +5611,7 @@
         <v>53</v>
       </c>
       <c r="AC23" s="7" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AD23" s="7">
         <v>4</v>
@@ -5728,16 +5728,16 @@
     </row>
     <row r="24" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A24" s="3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B24" s="3">
         <v>35</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="E24" s="3" t="s">
         <v>28</v>
@@ -5755,11 +5755,11 @@
         <v>109</v>
       </c>
       <c r="J24" s="3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="K24" s="3"/>
       <c r="L24" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M24" s="3">
         <v>40</v>
@@ -5810,7 +5810,7 @@
         <v>53</v>
       </c>
       <c r="AC24" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AD24" s="7">
         <v>3</v>
@@ -5927,19 +5927,19 @@
     </row>
     <row r="25" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A25" s="3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B25" s="3">
         <v>58</v>
       </c>
       <c r="C25" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="D25" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="D25" s="3" t="s">
-        <v>173</v>
-      </c>
       <c r="E25" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F25" s="3" t="s">
         <v>29</v>
@@ -5954,13 +5954,13 @@
         <v>100</v>
       </c>
       <c r="J25" s="3" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="K25" s="3">
         <v>1</v>
       </c>
       <c r="L25" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M25" s="3">
         <v>35</v>
@@ -6008,10 +6008,10 @@
         <v>54</v>
       </c>
       <c r="AB25" s="7" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="AC25" s="7" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AD25" s="7">
         <v>4</v>
@@ -6128,19 +6128,19 @@
     </row>
     <row r="26" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A26" s="3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B26" s="3">
         <v>57</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F26" s="3" t="s">
         <v>29</v>
@@ -6155,11 +6155,11 @@
         <v>111</v>
       </c>
       <c r="J26" s="3" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="K26" s="3"/>
       <c r="L26" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M26" s="3">
         <v>40</v>
@@ -6210,7 +6210,7 @@
         <v>53</v>
       </c>
       <c r="AC26" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AD26" s="7">
         <v>5</v>
@@ -6327,19 +6327,19 @@
     </row>
     <row r="27" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A27" s="3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B27" s="3">
         <v>29</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F27" s="3" t="s">
         <v>29</v>
@@ -6354,13 +6354,13 @@
         <v>112</v>
       </c>
       <c r="J27" s="3" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="K27" s="3">
         <v>8</v>
       </c>
       <c r="L27" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M27" s="3">
         <v>35</v>
@@ -6411,7 +6411,7 @@
         <v>53</v>
       </c>
       <c r="AC27" s="7" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AD27" s="7">
         <v>3</v>
@@ -6528,19 +6528,19 @@
     </row>
     <row r="28" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A28" s="3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B28" s="3">
         <v>67</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F28" s="3" t="s">
         <v>33</v>
@@ -6555,11 +6555,11 @@
         <v>59</v>
       </c>
       <c r="J28" s="3" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="K28" s="3"/>
       <c r="L28" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M28" s="3">
         <v>40</v>
@@ -6607,7 +6607,7 @@
         <v>27</v>
       </c>
       <c r="AC28" s="7" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AD28" s="7">
         <v>5</v>
@@ -6724,19 +6724,19 @@
     </row>
     <row r="29" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A29" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B29" s="3">
         <v>48</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F29" s="3" t="s">
         <v>33</v>
@@ -6751,13 +6751,13 @@
         <v>37</v>
       </c>
       <c r="J29" s="3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="K29" s="3">
         <v>5</v>
       </c>
       <c r="L29" s="12" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="M29" s="3">
         <v>56</v>
@@ -6805,7 +6805,7 @@
         <v>53</v>
       </c>
       <c r="AC29" s="7" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="AD29" s="7">
         <v>5</v>
@@ -6922,19 +6922,19 @@
     </row>
     <row r="30" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A30" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B30" s="3">
         <v>61</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="F30" s="3" t="s">
         <v>29</v>
@@ -6949,11 +6949,11 @@
         <v>38</v>
       </c>
       <c r="J30" s="3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="K30" s="3"/>
       <c r="L30" s="12" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="M30" s="3">
         <v>30</v>
@@ -6998,10 +6998,10 @@
         <v>54</v>
       </c>
       <c r="AB30" s="7" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="AC30" s="7" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AD30" s="7">
         <v>3</v>
@@ -7118,19 +7118,19 @@
     </row>
     <row r="31" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A31" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B31" s="3">
         <v>77</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D31" s="3" t="s">
         <v>46</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F31" t="s">
         <v>29</v>
@@ -7145,11 +7145,11 @@
         <v>47</v>
       </c>
       <c r="J31" s="3" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="K31" s="3"/>
       <c r="L31" s="12" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="M31" s="3">
         <v>60</v>
@@ -7197,10 +7197,10 @@
         <v>53</v>
       </c>
       <c r="AB31" s="7" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="AC31" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AD31" s="7">
         <v>5</v>
@@ -7317,16 +7317,16 @@
     </row>
     <row r="32" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A32" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B32" s="3">
         <v>36</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E32" s="3" t="s">
         <v>48</v>
@@ -7344,13 +7344,13 @@
         <v>35</v>
       </c>
       <c r="J32" s="3" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="K32" s="3">
         <v>4</v>
       </c>
       <c r="L32" s="12" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="M32" s="3">
         <v>70</v>
@@ -7401,7 +7401,7 @@
         <v>53</v>
       </c>
       <c r="AC32" s="7" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="AD32" s="7">
         <v>1</v>
@@ -7518,19 +7518,19 @@
     </row>
     <row r="33" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A33" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B33" s="3">
         <v>57</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="F33" s="3" t="s">
         <v>29</v>
@@ -7545,13 +7545,13 @@
         <v>49</v>
       </c>
       <c r="J33" s="3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="K33" s="3">
         <v>2</v>
       </c>
       <c r="L33" s="12" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="M33" s="3">
         <v>60</v>
@@ -7599,7 +7599,7 @@
         <v>53</v>
       </c>
       <c r="AC33" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AD33" s="7">
         <v>4</v>
@@ -7716,16 +7716,16 @@
     </row>
     <row r="34" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A34" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B34" s="3">
         <v>37</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="E34" s="3" t="s">
         <v>28</v>
@@ -7743,13 +7743,13 @@
         <v>50</v>
       </c>
       <c r="J34" s="3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="K34" s="3">
         <v>1</v>
       </c>
       <c r="L34" s="12" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="M34" s="4">
         <v>60</v>
@@ -7797,7 +7797,7 @@
         <v>53</v>
       </c>
       <c r="AC34" s="7" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AD34" s="7">
         <v>3</v>
@@ -7914,19 +7914,19 @@
     </row>
     <row r="35" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A35" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B35" s="3">
         <v>33</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F35" s="3" t="s">
         <v>29</v>
@@ -7941,13 +7941,13 @@
         <v>51</v>
       </c>
       <c r="J35" s="3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="K35" s="3">
         <v>3</v>
       </c>
       <c r="L35" s="5" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="M35" s="3">
         <v>60</v>
@@ -7995,7 +7995,7 @@
         <v>53</v>
       </c>
       <c r="AC35" s="7" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AD35" s="7">
         <v>3</v>
@@ -8112,16 +8112,16 @@
     </row>
     <row r="36" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A36" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B36" s="3">
         <v>65</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="E36" s="3" t="s">
         <v>28</v>
@@ -8139,11 +8139,11 @@
         <v>58</v>
       </c>
       <c r="J36" s="3" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="K36" s="3"/>
       <c r="L36" s="12" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="M36" s="3">
         <v>20</v>
@@ -8188,10 +8188,10 @@
         <v>53</v>
       </c>
       <c r="AB36" s="7" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="AC36" s="7" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AD36" s="7">
         <v>3</v>
@@ -8308,19 +8308,19 @@
     </row>
     <row r="37" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A37" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B37" s="3">
         <v>38</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="F37" s="3" t="s">
         <v>29</v>
@@ -8335,13 +8335,13 @@
         <v>59</v>
       </c>
       <c r="J37" s="3" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="K37" s="3">
         <v>1</v>
       </c>
       <c r="L37" s="5" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="M37" s="3">
         <v>45</v>
@@ -8392,7 +8392,7 @@
         <v>53</v>
       </c>
       <c r="AC37" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AD37" s="7">
         <v>5</v>
@@ -8509,16 +8509,16 @@
     </row>
     <row r="38" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A38" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B38" s="3">
         <v>27</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="E38" s="3" t="s">
         <v>48</v>
@@ -8536,13 +8536,13 @@
         <v>60</v>
       </c>
       <c r="J38" s="3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="K38" s="3">
         <v>2</v>
       </c>
       <c r="L38" s="12" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="M38" s="3">
         <v>50</v>
@@ -8593,7 +8593,7 @@
         <v>53</v>
       </c>
       <c r="AC38" s="7" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="AD38" s="7">
         <v>5</v>
@@ -8710,19 +8710,19 @@
     </row>
     <row r="39" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A39" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B39" s="3">
         <v>60</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="F39" s="3" t="s">
         <v>29</v>
@@ -8737,13 +8737,13 @@
         <v>51</v>
       </c>
       <c r="J39" s="3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="K39" s="3">
         <v>2</v>
       </c>
       <c r="L39" s="12" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="M39" s="3">
         <v>40</v>
@@ -8794,7 +8794,7 @@
         <v>53</v>
       </c>
       <c r="AC39" s="7" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="AD39" s="7">
         <v>5</v>
@@ -8911,16 +8911,16 @@
     </row>
     <row r="40" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A40" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B40" s="3">
         <v>58</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E40" s="3" t="s">
         <v>28</v>
@@ -8938,13 +8938,13 @@
         <v>63</v>
       </c>
       <c r="J40" s="3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="K40" s="3">
         <v>3</v>
       </c>
       <c r="L40" s="12" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="M40" s="3">
         <v>60</v>
@@ -8989,10 +8989,10 @@
         <v>54</v>
       </c>
       <c r="AB40" s="7" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AC40" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AD40" s="7">
         <v>3</v>
@@ -9109,19 +9109,19 @@
     </row>
     <row r="41" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A41" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B41" s="3">
         <v>65</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F41" s="3" t="s">
         <v>29</v>
@@ -9136,13 +9136,13 @@
         <v>67</v>
       </c>
       <c r="J41" s="3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="K41" s="3">
         <v>3</v>
       </c>
       <c r="L41" s="12" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="M41" s="3">
         <v>50</v>
@@ -9187,10 +9187,10 @@
         <v>54</v>
       </c>
       <c r="AB41" s="7" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="AC41" s="7" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AD41" s="7">
         <v>3</v>
@@ -9307,19 +9307,19 @@
     </row>
     <row r="42" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A42" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B42" s="3">
         <v>41</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F42" s="3" t="s">
         <v>29</v>
@@ -9334,11 +9334,11 @@
         <v>70</v>
       </c>
       <c r="J42" s="3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="K42" s="3"/>
       <c r="L42" s="12" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="M42" s="3">
         <v>56</v>
@@ -9389,7 +9389,7 @@
         <v>53</v>
       </c>
       <c r="AC42" s="7" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AD42" s="7">
         <v>3</v>
@@ -9506,19 +9506,19 @@
     </row>
     <row r="43" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A43" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B43" s="3">
         <v>47</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F43" s="3" t="s">
         <v>74</v>
@@ -9533,13 +9533,13 @@
         <v>73</v>
       </c>
       <c r="J43" s="3" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="K43" s="3">
         <v>4</v>
       </c>
       <c r="L43" s="12" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="M43" s="3">
         <v>18</v>
@@ -9584,10 +9584,10 @@
         <v>54</v>
       </c>
       <c r="AB43" s="7" t="s">
+        <v>205</v>
+      </c>
+      <c r="AC43" s="7" t="s">
         <v>206</v>
-      </c>
-      <c r="AC43" s="7" t="s">
-        <v>207</v>
       </c>
       <c r="AD43" s="7">
         <v>3</v>
@@ -9704,19 +9704,19 @@
     </row>
     <row r="44" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A44" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B44" s="3">
         <v>29</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D44" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="E44" s="3" t="s">
         <v>176</v>
-      </c>
-      <c r="E44" s="3" t="s">
-        <v>177</v>
       </c>
       <c r="F44" s="3" t="s">
         <v>33</v>
@@ -9731,13 +9731,13 @@
         <v>78</v>
       </c>
       <c r="J44" s="3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="K44" s="3">
         <v>6</v>
       </c>
       <c r="L44" s="12" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="M44" s="4">
         <v>44</v>
@@ -9785,7 +9785,7 @@
         <v>53</v>
       </c>
       <c r="AC44" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AD44" s="7">
         <v>4</v>
@@ -9902,19 +9902,19 @@
     </row>
     <row r="45" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A45" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B45" s="3">
         <v>18</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F45" s="3" t="s">
         <v>29</v>
@@ -9929,11 +9929,11 @@
         <v>50</v>
       </c>
       <c r="J45" s="3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="K45" s="3"/>
       <c r="L45" s="12" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="M45" s="3">
         <v>40</v>
@@ -9984,7 +9984,7 @@
         <v>53</v>
       </c>
       <c r="AC45" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AD45" s="7">
         <v>5</v>

</xml_diff>